<commit_message>
Add second easy daily round
</commit_message>
<xml_diff>
--- a/exports/daily-games.xlsx
+++ b/exports/daily-games.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Games" sheetId="1" r:id="R54bb49ae13584e77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Games" sheetId="1" r:id="Rbed25c0477c346aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -332,7 +332,7 @@
         <x:v>q2_borough</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>q3_medium</x:v>
+        <x:v>q3_easy</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
         <x:v>q3_borough</x:v>
@@ -367,28 +367,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D2" s="7" t="str">
-        <x:v>B &amp; B Carousell</x:v>
+        <x:v>Forest Park Carousel</x:v>
       </x:c>
       <x:c r="E2" s="7" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F2" s="7" t="str">
-        <x:v>Beth Olam Cemetery</x:v>
+        <x:v>Rainey Memorial Gates</x:v>
       </x:c>
       <x:c r="G2" s="7" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H2" s="7" t="str">
-        <x:v>Middletown Plaza</x:v>
+        <x:v>Jacques Marchais Center of Tibetan Art</x:v>
       </x:c>
       <x:c r="I2" s="7" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J2" s="7" t="str">
-        <x:v>Gardiner-Tyler House</x:v>
+        <x:v>Old Stone House of Brooklyn</x:v>
       </x:c>
       <x:c r="K2" s="7" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="L2" s="15" t="str">
         <x:v>scheduled</x:v>
@@ -406,28 +406,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Forest Park Carousel</x:v>
+        <x:v>Litchfield Villa</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>Boys' High School</x:v>
+        <x:v>Alice Austen House</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
-        <x:v>United Workers' Cooperatives</x:v>
+        <x:v>Astoria Center of Israel</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="J3" s="9" t="str">
-        <x:v>Billou-Stillwell-Perine House</x:v>
+        <x:v>St. James' Episcopal Church and Parish House</x:v>
       </x:c>
       <x:c r="K3" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L3" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -445,28 +445,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Ridgewood Reservoir</x:v>
+        <x:v>Brooklyn Public Library</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>Staten Island Light</x:v>
+        <x:v>Williamsbridge Oval Park</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Jamaica Chamber of Commerce Building</x:v>
+        <x:v>Richmond Terrace Cemeteries</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J4" s="9" t="str">
-        <x:v>St. James' Episcopal Church and Parish House</x:v>
+        <x:v>New York Architectural Terra Cotta Company Office Building</x:v>
       </x:c>
       <x:c r="K4" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L4" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -484,28 +484,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Garibaldi Memorial</x:v>
+        <x:v>Brooklyn Borough Hall</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>Manhattan Beach Jewish Center</x:v>
+        <x:v>Conference House</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Kurtz, J., and Sons Store Building</x:v>
+        <x:v>Bronx Borough Courthouse</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
-        <x:v>Hall of Fame Complex</x:v>
+        <x:v>Allen-Beville House</x:v>
       </x:c>
       <x:c r="K5" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L5" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -523,25 +523,25 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
+        <x:v>Federal Hall National Memorial</x:v>
+      </x:c>
+      <x:c r="E6" s="9" t="str">
+        <x:v>Manhattan</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
         <x:v>Jerome Park Reservoir</x:v>
       </x:c>
-      <x:c r="E6" s="9" t="str">
-        <x:v>The Bronx</x:v>
-      </x:c>
-      <x:c r="F6" s="9" t="str">
-        <x:v>University Settlement House</x:v>
-      </x:c>
       <x:c r="G6" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:v>Sylvan Grove Cemetery</x:v>
+        <x:v>Staten Island Light</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
         <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>New York Architectural Terra Cotta Company Office Building</x:v>
+        <x:v>Flushing Armory</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
         <x:v>Queens</x:v>
@@ -562,25 +562,25 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
+        <x:v>Marine Air Terminal, La Guardia Airport</x:v>
+      </x:c>
+      <x:c r="E7" s="9" t="str">
+        <x:v>Queens</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
         <x:v>Bartow-Pell Mansion and Carriage House</x:v>
       </x:c>
-      <x:c r="E7" s="9" t="str">
-        <x:v>The Bronx</x:v>
-      </x:c>
-      <x:c r="F7" s="9" t="str">
-        <x:v>Quarters A</x:v>
-      </x:c>
       <x:c r="G7" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
-        <x:v>Office of the Register</x:v>
+        <x:v>Erasmus Hall Academy</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
-        <x:v>Frederick Law Olmsted Sr. Farmhouse</x:v>
+        <x:v>Gardiner-Tyler House</x:v>
       </x:c>
       <x:c r="K7" s="9" t="str">
         <x:v>Staten Island</x:v>
@@ -601,28 +601,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Loew's Kameo Theater</x:v>
+        <x:v>Washington Bridge</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>Saxe Embroidery Company Building</x:v>
+        <x:v>Battery Weed</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>Kingsland Homestead</x:v>
+        <x:v>Jewish Center of Coney Island</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>Moore-McMillen House</x:v>
+        <x:v>Spear &amp; Company Factory</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L8" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -640,28 +640,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Old Town of Flushing Burial Ground</x:v>
+        <x:v>Port Morris Ferry Bridges</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Wyckoff-Bennett Homestead</x:v>
+        <x:v>Ridgewood Reservoir</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str">
-        <x:v>Fire Fighter</x:v>
+        <x:v>Beth Olam Cemetery</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
-        <x:v>Hertlein and Schlatter Silk Trimmings Factory</x:v>
+        <x:v>Billou-Stillwell-Perine House</x:v>
       </x:c>
       <x:c r="K9" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L9" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -679,28 +679,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Conference House</x:v>
+        <x:v>Woodlawn Cemetery</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>Gage and Tollner Restaurant</x:v>
+        <x:v>Sailors' Snug Harbor</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
-        <x:v>Fort Totten Officers' Club</x:v>
+        <x:v>Kurtz, J., and Sons Store Building</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>Dodge, William E., House</x:v>
+        <x:v>Lincoln Club</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="L10" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -718,25 +718,25 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>Battery Weed</x:v>
+        <x:v>Old Quaker Meetinghouse</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>New Lots Reformed Church and Cemetery</x:v>
+        <x:v>Floyd Bennett Field</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str">
-        <x:v>Kent Manor</x:v>
+        <x:v>New Dorp Light</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>Valentine-Varian House</x:v>
+        <x:v>Hall of Fame Complex</x:v>
       </x:c>
       <x:c r="K11" s="9" t="str">
         <x:v>The Bronx</x:v>
@@ -757,28 +757,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Theodore Roosevelt Birthplace</x:v>
+        <x:v>Biltmore Theater</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
-        <x:v>Sage, Russell, Memorial Church</x:v>
+        <x:v>King Manor</x:v>
       </x:c>
       <x:c r="G12" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="H12" s="9" t="str">
-        <x:v>Eighth Regiment Armory (Kingsbridge Armory)</x:v>
+        <x:v>Silver Lake Cemetery</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
-        <x:v>Kreischer House</x:v>
+        <x:v>Hertlein and Schlatter Silk Trimmings Factory</x:v>
       </x:c>
       <x:c r="K12" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L12" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -796,28 +796,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>African Burial Ground</x:v>
+        <x:v>New Amsterdam Theater</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
-        <x:v>Trinity Chapel</x:v>
+        <x:v>Edgar Allan Poe Cottage</x:v>
       </x:c>
       <x:c r="G13" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H13" s="9" t="str">
-        <x:v>Edgewater Village Hall and Tappen Park</x:v>
+        <x:v>Benevolent and Protective Order of Elks, Lodge #878</x:v>
       </x:c>
       <x:c r="I13" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="J13" s="9" t="str">
-        <x:v>Grace Episcopal Church</x:v>
+        <x:v>Frederick Law Olmsted Sr. Farmhouse</x:v>
       </x:c>
       <x:c r="K13" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L13" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -835,28 +835,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
-        <x:v>Fort Wadsworth</x:v>
+        <x:v>Green-Wood Cemetery</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F14" s="9" t="str">
-        <x:v>Beth-El Jewish Center of Flatbush</x:v>
+        <x:v>Garibaldi Memorial</x:v>
       </x:c>
       <x:c r="G14" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H14" s="9" t="str">
-        <x:v>Maple Grove Cemetery</x:v>
+        <x:v>Casita Rincon Criollo</x:v>
       </x:c>
       <x:c r="I14" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J14" s="9" t="str">
-        <x:v>Riverdale Presbyterian Church Complex</x:v>
+        <x:v>Cornell Farmhouse</x:v>
       </x:c>
       <x:c r="K14" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L14" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -874,25 +874,25 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>Alice Austen House</x:v>
+        <x:v>Morris–Jumel Mansion</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str">
-        <x:v>Riverside Park and Drive</x:v>
+        <x:v>Fort Tompkins Quadrangle</x:v>
       </x:c>
       <x:c r="G15" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H15" s="9" t="str">
-        <x:v>Rockaway Courthouse</x:v>
+        <x:v>Trinity Chapel</x:v>
       </x:c>
       <x:c r="I15" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J15" s="9" t="str">
-        <x:v>C. Rieger's Sons Factory</x:v>
+        <x:v>Dodge, William E., House</x:v>
       </x:c>
       <x:c r="K15" s="9" t="str">
         <x:v>The Bronx</x:v>
@@ -913,28 +913,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>Old Orchard Shoal Light Station</x:v>
+        <x:v>Ocean Parkway</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F16" s="9" t="str">
-        <x:v>Alku &amp; Alku Toinen</x:v>
+        <x:v>Wave Hill</x:v>
       </x:c>
       <x:c r="G16" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H16" s="9" t="str">
-        <x:v>BOHEMIAN HALL AND PARK</x:v>
+        <x:v>First Reformed Church of College Point</x:v>
       </x:c>
       <x:c r="I16" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J16" s="9" t="str">
-        <x:v>Reformed Church of Melrose</x:v>
+        <x:v>Moore-McMillen House</x:v>
       </x:c>
       <x:c r="K16" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L16" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -958,22 +958,22 @@
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F17" s="9" t="str">
-        <x:v>Old Brooklyn Fire Headquarters</x:v>
+        <x:v>Prospect Park Boathouse</x:v>
       </x:c>
       <x:c r="G17" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H17" s="9" t="str">
-        <x:v>Silver Lake Cemetery</x:v>
+        <x:v>Flushing High School</x:v>
       </x:c>
       <x:c r="I17" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="J17" s="9" t="str">
-        <x:v>Allen-Beville House</x:v>
+        <x:v>Kreischer House</x:v>
       </x:c>
       <x:c r="K17" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L17" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -991,25 +991,25 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>Floyd Bennett Field</x:v>
+        <x:v>Fort Wadsworth</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="F18" s="9" t="str">
-        <x:v>Wyckoff-Snediker Family Cemetery</x:v>
+        <x:v>Steinway House</x:v>
       </x:c>
       <x:c r="G18" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="H18" s="9" t="str">
-        <x:v>St. Paul's Memorial Church and Rectory</x:v>
+        <x:v>Nassau Brewery</x:v>
       </x:c>
       <x:c r="I18" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J18" s="9" t="str">
-        <x:v>St. Anselm's Roman Catholic Church Complex</x:v>
+        <x:v>Valentine-Varian House</x:v>
       </x:c>
       <x:c r="K18" s="9" t="str">
         <x:v>The Bronx</x:v>
@@ -1030,28 +1030,28 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>Port Morris Ferry Bridges</x:v>
+        <x:v>The Public Theater</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F19" s="9" t="str">
-        <x:v>Park Row Building</x:v>
+        <x:v>Ward, Caleb T., Mansion</x:v>
       </x:c>
       <x:c r="G19" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H19" s="9" t="str">
-        <x:v>Talmud Torah Atereth Israel</x:v>
+        <x:v>Brooklyn Trust Company</x:v>
       </x:c>
       <x:c r="I19" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J19" s="9" t="str">
-        <x:v>LaTourette House</x:v>
+        <x:v>Grace Episcopal Church</x:v>
       </x:c>
       <x:c r="K19" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L19" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1069,28 +1069,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>Fort Tompkins Quadrangle</x:v>
+        <x:v>Gracie Mansion</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
-        <x:v>Whitney Museum of American Art</x:v>
+        <x:v>Rego Park Jewish Center</x:v>
       </x:c>
       <x:c r="G20" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H20" s="9" t="str">
-        <x:v>The Church-in-the-Gardens</x:v>
+        <x:v>United Workers' Cooperatives</x:v>
       </x:c>
       <x:c r="I20" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J20" s="9" t="str">
-        <x:v>Spaulding, Henry F., Coachman's House</x:v>
+        <x:v>LaTourette House</x:v>
       </x:c>
       <x:c r="K20" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L20" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1108,28 +1108,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>King Manor</x:v>
+        <x:v>Riverside Park and Drive</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F21" s="9" t="str">
-        <x:v>Verdi, Giuseppe, Monument</x:v>
+        <x:v>Voorlezer's House</x:v>
       </x:c>
       <x:c r="G21" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H21" s="9" t="str">
-        <x:v>St. Peter's Church, Chapel and Cemetery Complex</x:v>
+        <x:v>Bronx County Courthouse</x:v>
       </x:c>
       <x:c r="I21" s="9" t="str">
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J21" s="9" t="str">
-        <x:v>Boardman- Mitchell House</x:v>
+        <x:v>Trinity Lutheran Church</x:v>
       </x:c>
       <x:c r="K21" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L21" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1147,25 +1147,25 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>Flushing Town Hall</x:v>
+        <x:v>Loew's Kameo Theater</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
-        <x:v>Young Israel of Flatbush</x:v>
+        <x:v>Parkway Village</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H22" s="9" t="str">
-        <x:v>Riverdale, Spuyten Duyvil, Kingsbridge Memorial Bell Tower</x:v>
+        <x:v>St. Peter's Church, Chapel and Cemetery Complex</x:v>
       </x:c>
       <x:c r="I22" s="9" t="str">
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J22" s="9" t="str">
-        <x:v>McFarlane-Bredt House</x:v>
+        <x:v>Boardman- Mitchell House</x:v>
       </x:c>
       <x:c r="K22" s="9" t="str">
         <x:v>Staten Island</x:v>
@@ -1186,28 +1186,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>Ocean Parkway Jewish Center</x:v>
+        <x:v>McGolrick, Monsignor, Park and Shelter Pavilion</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F23" s="9" t="str">
-        <x:v>Richmond Terrace Cemeteries</x:v>
+        <x:v>Old Town of Flushing Burial Ground</x:v>
       </x:c>
       <x:c r="G23" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H23" s="9" t="str">
-        <x:v>Casa Amadeo, antigua Casa Hernandez</x:v>
+        <x:v>West Bank Light Station</x:v>
       </x:c>
       <x:c r="I23" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J23" s="9" t="str">
-        <x:v>Flushing Armory</x:v>
+        <x:v>Riverdale Presbyterian Church Complex</x:v>
       </x:c>
       <x:c r="K23" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L23" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1225,28 +1225,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>Woodlawn Cemetery</x:v>
+        <x:v>Eastern Parkway</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F24" s="9" t="str">
-        <x:v>Prospect Park Boathouse</x:v>
+        <x:v>RKO Keith's Theater</x:v>
       </x:c>
       <x:c r="G24" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
-        <x:v>West Bank Light Station</x:v>
+        <x:v>Keeper's House, Williamsbridge Reservoir</x:v>
       </x:c>
       <x:c r="I24" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J24" s="9" t="str">
-        <x:v>Spear &amp; Company Factory</x:v>
+        <x:v>McFarlane-Bredt House</x:v>
       </x:c>
       <x:c r="K24" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L24" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1264,28 +1264,28 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>New York Public Library</x:v>
+        <x:v>Theodore Roosevelt Birthplace</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F25" s="9" t="str">
-        <x:v>Joralemon Street Tunnel (IRT)</x:v>
+        <x:v>Loew's King Theatre</x:v>
       </x:c>
       <x:c r="G25" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H25" s="9" t="str">
-        <x:v>Bronx Borough Courthouse</x:v>
+        <x:v>Ward's Point Conservation Area</x:v>
       </x:c>
       <x:c r="I25" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J25" s="9" t="str">
-        <x:v>Kreuzer-Pelton House</x:v>
+        <x:v>C. Rieger's Sons Factory</x:v>
       </x:c>
       <x:c r="K25" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L25" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1303,28 +1303,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>Old Quaker Meetinghouse</x:v>
+        <x:v>Crotona Play Center</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F26" s="9" t="str">
-        <x:v>Friends Meetinghouse and School</x:v>
+        <x:v>Parkway Theater</x:v>
       </x:c>
       <x:c r="G26" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H26" s="9" t="str">
-        <x:v>Vanderbilt Family Cemetery and Mausoleum</x:v>
+        <x:v>Maple Grove Cemetery</x:v>
       </x:c>
       <x:c r="I26" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="J26" s="9" t="str">
-        <x:v>St. Ann's Church Complex</x:v>
+        <x:v>Kreuzer-Pelton House</x:v>
       </x:c>
       <x:c r="K26" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L26" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1342,22 +1342,22 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>Washington Bridge</x:v>
+        <x:v>Jeffrey's Hook Lighthouse</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F27" s="9" t="str">
-        <x:v>Charlie Parker Residence</x:v>
+        <x:v>Flushing Town Hall</x:v>
       </x:c>
       <x:c r="G27" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H27" s="9" t="str">
-        <x:v>La Casina</x:v>
+        <x:v>Boston Road Plaza</x:v>
       </x:c>
       <x:c r="I27" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J27" s="9" t="str">
         <x:v>Immanuel Union Church</x:v>
@@ -1381,19 +1381,19 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>Rainey Memorial Gates</x:v>
+        <x:v>B &amp; B Carousell</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F28" s="9" t="str">
-        <x:v>Old Gravesend Cemetery</x:v>
+        <x:v>Fort Schuyler</x:v>
       </x:c>
       <x:c r="G28" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H28" s="9" t="str">
-        <x:v>Benevolent and Protective Order of Elks, Lodge #878</x:v>
+        <x:v>Queens County Savings Bank, Kew Gardens Hills Branch</x:v>
       </x:c>
       <x:c r="I28" s="9" t="str">
         <x:v>Queens</x:v>
@@ -1420,28 +1420,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>Steinway House</x:v>
+        <x:v>U.S. Army Military Ocean Terminal</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F29" s="9" t="str">
-        <x:v>Erasmus Hall Academy</x:v>
+        <x:v>Old Orchard Shoal Light Station</x:v>
       </x:c>
       <x:c r="G29" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H29" s="9" t="str">
-        <x:v>Bronx County Courthouse</x:v>
+        <x:v>Office of the Register</x:v>
       </x:c>
       <x:c r="I29" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="J29" s="9" t="str">
-        <x:v>Louis A. and Laura Stirn House</x:v>
+        <x:v>Reformed Church of Melrose</x:v>
       </x:c>
       <x:c r="K29" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L29" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1459,28 +1459,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>Wave Hill</x:v>
+        <x:v>Ocean Parkway Jewish Center</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F30" s="9" t="str">
-        <x:v>Fiorentino Plaza</x:v>
+        <x:v>Staten Island Ferry Terminal</x:v>
       </x:c>
       <x:c r="G30" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H30" s="9" t="str">
-        <x:v>Astoria Center of Israel</x:v>
+        <x:v>Long Island City Courthouse Complex</x:v>
       </x:c>
       <x:c r="I30" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J30" s="9" t="str">
-        <x:v>Old Stone House of Brooklyn</x:v>
+        <x:v>St. Anselm's Roman Catholic Church Complex</x:v>
       </x:c>
       <x:c r="K30" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L30" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1498,28 +1498,28 @@
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>Trinity Church and Graveyard</x:v>
+        <x:v>African Burial Ground</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F31" s="9" t="str">
-        <x:v>Jewish Center of Kings Highway</x:v>
+        <x:v>Long Island Motor Parkway</x:v>
       </x:c>
       <x:c r="G31" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H31" s="9" t="str">
-        <x:v>Jacques Marchais Center of Tibetan Art</x:v>
+        <x:v>Mary A. Whalen</x:v>
       </x:c>
       <x:c r="I31" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J31" s="9" t="str">
-        <x:v>Cornell Farmhouse</x:v>
+        <x:v>Louis A. and Laura Stirn House</x:v>
       </x:c>
       <x:c r="K31" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L31" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1537,28 +1537,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>Brooklyn Public Library</x:v>
+        <x:v>Ed Sullivan Theater</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F32" s="9" t="str">
-        <x:v>Flushing High School</x:v>
+        <x:v>Hamilton Grange National Memorial</x:v>
       </x:c>
       <x:c r="G32" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H32" s="9" t="str">
-        <x:v>Sunnyslope</x:v>
+        <x:v>Casemate Fort, Whiting Quadrangle</x:v>
       </x:c>
       <x:c r="I32" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J32" s="9" t="str">
-        <x:v>Circle Line X</x:v>
+        <x:v>Conrad Voelcker House</x:v>
       </x:c>
       <x:c r="K32" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L32" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1576,28 +1576,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>Fort Schuyler</x:v>
+        <x:v>New York Public Library</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F33" s="9" t="str">
-        <x:v>Public Bath No. 7</x:v>
+        <x:v>Morgan Library</x:v>
       </x:c>
       <x:c r="G33" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H33" s="9" t="str">
-        <x:v>First Reformed Church of College Point</x:v>
+        <x:v>Beth-El Jewish Center of Flatbush</x:v>
       </x:c>
       <x:c r="I33" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J33" s="9" t="str">
-        <x:v>Corbin Building</x:v>
+        <x:v>Sohmer Piano Factory</x:v>
       </x:c>
       <x:c r="K33" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L33" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1615,25 +1615,25 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>Loew's King Theatre</x:v>
+        <x:v>Trinity Church and Graveyard</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F34" s="9" t="str">
-        <x:v>Admiral David Glasgow Farragut Gravesite</x:v>
+        <x:v>Castle Clinton National Monument</x:v>
       </x:c>
       <x:c r="G34" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H34" s="9" t="str">
-        <x:v>Staten Island Borough Hall and Richmond County Courthouse</x:v>
+        <x:v>Gage and Tollner Restaurant</x:v>
       </x:c>
       <x:c r="I34" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J34" s="9" t="str">
-        <x:v>Trinity Lutheran Church</x:v>
+        <x:v>Saint James Church</x:v>
       </x:c>
       <x:c r="K34" s="9" t="str">
         <x:v>Queens</x:v>
@@ -1654,25 +1654,25 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>RKO Keith's Theater</x:v>
+        <x:v>Queensboro Bridge</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F35" s="9" t="str">
-        <x:v>Brooklyn Historical Society Building</x:v>
+        <x:v>American Stock Exchange</x:v>
       </x:c>
       <x:c r="G35" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H35" s="9" t="str">
-        <x:v>Ward's Point Conservation Area</x:v>
+        <x:v>Joralemon Street Tunnel (IRT)</x:v>
       </x:c>
       <x:c r="I35" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J35" s="9" t="str">
-        <x:v>Christ Church Complex</x:v>
+        <x:v>Spaulding, Henry F., Coachman's House</x:v>
       </x:c>
       <x:c r="K35" s="9" t="str">
         <x:v>The Bronx</x:v>
@@ -1693,28 +1693,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D36" s="11" t="str">
-        <x:v>McGolrick, Monsignor, Park and Shelter Pavilion</x:v>
+        <x:v>Whitney Museum of American Art</x:v>
       </x:c>
       <x:c r="E36" s="11" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F36" s="11" t="str">
-        <x:v>Queens County Savings Bank, Kew Gardens Hills Branch</x:v>
+        <x:v>College of the City of New York</x:v>
       </x:c>
       <x:c r="G36" s="11" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H36" s="11" t="str">
-        <x:v>Lorillard Snuff Mill</x:v>
+        <x:v>Jewish Center of Kings Highway</x:v>
       </x:c>
       <x:c r="I36" s="11" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J36" s="11" t="str">
-        <x:v>Bayard Rustin Apartment</x:v>
+        <x:v>Jamaica Savings Bank</x:v>
       </x:c>
       <x:c r="K36" s="11" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L36" s="17" t="str">
         <x:v>scheduled</x:v>

</xml_diff>

<commit_message>
Rebrand daily difficulty tiers
</commit_message>
<xml_diff>
--- a/exports/daily-games.xlsx
+++ b/exports/daily-games.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Games" sheetId="1" r:id="Rbed25c0477c346aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Games" sheetId="1" r:id="R01871f8d06cd49fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -320,31 +320,31 @@
         <x:v>date</x:v>
       </x:c>
       <x:c r="B1" s="4" t="str">
-        <x:v>q1_very_easy</x:v>
+        <x:v>q1_easy</x:v>
       </x:c>
       <x:c r="C1" s="4" t="str">
         <x:v>q1_borough</x:v>
       </x:c>
       <x:c r="D1" s="4" t="str">
-        <x:v>q2_easy</x:v>
+        <x:v>q2_medium</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
         <x:v>q2_borough</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>q3_easy</x:v>
+        <x:v>q3_medium</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
         <x:v>q3_borough</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>q4_medium</x:v>
+        <x:v>q4_hard</x:v>
       </x:c>
       <x:c r="I1" s="4" t="str">
         <x:v>q4_borough</x:v>
       </x:c>
       <x:c r="J1" s="4" t="str">
-        <x:v>q5_hard</x:v>
+        <x:v>q5_im_walking_here</x:v>
       </x:c>
       <x:c r="K1" s="4" t="str">
         <x:v>q5_borough</x:v>
@@ -385,10 +385,10 @@
         <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J2" s="7" t="str">
-        <x:v>Old Stone House of Brooklyn</x:v>
+        <x:v>New York Architectural Terra Cotta Company Office Building</x:v>
       </x:c>
       <x:c r="K2" s="7" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L2" s="15" t="str">
         <x:v>scheduled</x:v>
@@ -406,16 +406,16 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D3" s="9" t="str">
-        <x:v>Litchfield Villa</x:v>
+        <x:v>Federal Hall National Memorial</x:v>
       </x:c>
       <x:c r="E3" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F3" s="9" t="str">
-        <x:v>Alice Austen House</x:v>
+        <x:v>Biltmore Theater</x:v>
       </x:c>
       <x:c r="G3" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H3" s="9" t="str">
         <x:v>Astoria Center of Israel</x:v>
@@ -424,10 +424,10 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J3" s="9" t="str">
-        <x:v>St. James' Episcopal Church and Parish House</x:v>
+        <x:v>Old Stone House of Brooklyn</x:v>
       </x:c>
       <x:c r="K3" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="L3" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -445,28 +445,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
-        <x:v>Brooklyn Public Library</x:v>
+        <x:v>Litchfield Villa</x:v>
       </x:c>
       <x:c r="E4" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F4" s="9" t="str">
-        <x:v>Williamsbridge Oval Park</x:v>
+        <x:v>Alice Austen House</x:v>
       </x:c>
       <x:c r="G4" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H4" s="9" t="str">
-        <x:v>Richmond Terrace Cemeteries</x:v>
+        <x:v>Bronx Borough Courthouse</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J4" s="9" t="str">
-        <x:v>New York Architectural Terra Cotta Company Office Building</x:v>
+        <x:v>Circle Line X</x:v>
       </x:c>
       <x:c r="K4" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L4" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -484,28 +484,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Brooklyn Borough Hall</x:v>
+        <x:v>Brooklyn Public Library</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
-        <x:v>Conference House</x:v>
+        <x:v>Williamsbridge Oval Park</x:v>
       </x:c>
       <x:c r="G5" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>Bronx Borough Courthouse</x:v>
+        <x:v>Richmond Terrace Cemeteries</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
-        <x:v>Allen-Beville House</x:v>
+        <x:v>St. James' Episcopal Church and Parish House</x:v>
       </x:c>
       <x:c r="K5" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L5" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -523,28 +523,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D6" s="9" t="str">
-        <x:v>Federal Hall National Memorial</x:v>
+        <x:v>New Amsterdam Theater</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
-        <x:v>Jerome Park Reservoir</x:v>
+        <x:v>Brooklyn Borough Hall</x:v>
       </x:c>
       <x:c r="G6" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:v>Staten Island Light</x:v>
+        <x:v>Erasmus Hall Academy</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>Flushing Armory</x:v>
+        <x:v>Gardiner-Tyler House</x:v>
       </x:c>
       <x:c r="K6" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L6" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -562,28 +562,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D7" s="9" t="str">
-        <x:v>Marine Air Terminal, La Guardia Airport</x:v>
+        <x:v>Conference House</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
-        <x:v>Bartow-Pell Mansion and Carriage House</x:v>
+        <x:v>Jerome Park Reservoir</x:v>
       </x:c>
       <x:c r="G7" s="9" t="str">
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
-        <x:v>Erasmus Hall Academy</x:v>
+        <x:v>Staten Island Light</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
-        <x:v>Gardiner-Tyler House</x:v>
+        <x:v>Allen-Beville House</x:v>
       </x:c>
       <x:c r="K7" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L7" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -601,16 +601,16 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Washington Bridge</x:v>
+        <x:v>Morris–Jumel Mansion</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
-        <x:v>Battery Weed</x:v>
+        <x:v>Marine Air Terminal, La Guardia Airport</x:v>
       </x:c>
       <x:c r="G8" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
         <x:v>Jewish Center of Coney Island</x:v>
@@ -619,10 +619,10 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>Spear &amp; Company Factory</x:v>
+        <x:v>Billou-Stillwell-Perine House</x:v>
       </x:c>
       <x:c r="K8" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L8" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -640,16 +640,16 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>Port Morris Ferry Bridges</x:v>
+        <x:v>Bartow-Pell Mansion and Carriage House</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
-        <x:v>Ridgewood Reservoir</x:v>
+        <x:v>Washington Bridge</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str">
         <x:v>Beth Olam Cemetery</x:v>
@@ -658,10 +658,10 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
-        <x:v>Billou-Stillwell-Perine House</x:v>
+        <x:v>Hall of Fame Complex</x:v>
       </x:c>
       <x:c r="K9" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L9" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -679,13 +679,13 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>Woodlawn Cemetery</x:v>
+        <x:v>Port Morris Ferry Bridges</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>Sailors' Snug Harbor</x:v>
+        <x:v>Battery Weed</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
         <x:v>Staten Island</x:v>
@@ -697,10 +697,10 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>Lincoln Club</x:v>
+        <x:v>Frederick Law Olmsted Sr. Farmhouse</x:v>
       </x:c>
       <x:c r="K10" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L10" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -718,28 +718,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>Old Quaker Meetinghouse</x:v>
+        <x:v>Ridgewood Reservoir</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
-        <x:v>Floyd Bennett Field</x:v>
+        <x:v>Woodlawn Cemetery</x:v>
       </x:c>
       <x:c r="G11" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str">
-        <x:v>New Dorp Light</x:v>
+        <x:v>Nassau Brewery</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>Hall of Fame Complex</x:v>
+        <x:v>Corbin Building</x:v>
       </x:c>
       <x:c r="K11" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L11" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -757,28 +757,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>Biltmore Theater</x:v>
+        <x:v>Sailors' Snug Harbor</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
-        <x:v>King Manor</x:v>
+        <x:v>The Public Theater</x:v>
       </x:c>
       <x:c r="G12" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H12" s="9" t="str">
-        <x:v>Silver Lake Cemetery</x:v>
+        <x:v>Duke, James B., Mansion</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
-        <x:v>Hertlein and Schlatter Silk Trimmings Factory</x:v>
+        <x:v>Bayard Rustin Apartment</x:v>
       </x:c>
       <x:c r="K12" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L12" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -796,16 +796,16 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
-        <x:v>New Amsterdam Theater</x:v>
+        <x:v>Old Quaker Meetinghouse</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F13" s="9" t="str">
-        <x:v>Edgar Allan Poe Cottage</x:v>
+        <x:v>Floyd Bennett Field</x:v>
       </x:c>
       <x:c r="G13" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H13" s="9" t="str">
         <x:v>Benevolent and Protective Order of Elks, Lodge #878</x:v>
@@ -814,10 +814,10 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J13" s="9" t="str">
-        <x:v>Frederick Law Olmsted Sr. Farmhouse</x:v>
+        <x:v>Bell Telephone Laboratories</x:v>
       </x:c>
       <x:c r="K13" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L13" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -835,28 +835,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
+        <x:v>Gracie Mansion</x:v>
+      </x:c>
+      <x:c r="E14" s="9" t="str">
+        <x:v>Manhattan</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="str">
         <x:v>Green-Wood Cemetery</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="str">
-        <x:v>Brooklyn</x:v>
-      </x:c>
-      <x:c r="F14" s="9" t="str">
-        <x:v>Garibaldi Memorial</x:v>
-      </x:c>
       <x:c r="G14" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H14" s="9" t="str">
-        <x:v>Casita Rincon Criollo</x:v>
+        <x:v>Harlem Courthouse</x:v>
       </x:c>
       <x:c r="I14" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J14" s="9" t="str">
-        <x:v>Cornell Farmhouse</x:v>
+        <x:v>Hertlein and Schlatter Silk Trimmings Factory</x:v>
       </x:c>
       <x:c r="K14" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L14" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -874,28 +874,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D15" s="9" t="str">
-        <x:v>Morris–Jumel Mansion</x:v>
+        <x:v>King Manor</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F15" s="9" t="str">
-        <x:v>Fort Tompkins Quadrangle</x:v>
+        <x:v>Edgar Allan Poe Cottage</x:v>
       </x:c>
       <x:c r="G15" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H15" s="9" t="str">
-        <x:v>Trinity Chapel</x:v>
+        <x:v>Brooklyn Trust Company</x:v>
       </x:c>
       <x:c r="I15" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J15" s="9" t="str">
-        <x:v>Dodge, William E., House</x:v>
+        <x:v>Daily News Building</x:v>
       </x:c>
       <x:c r="K15" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L15" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -913,28 +913,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D16" s="9" t="str">
-        <x:v>Ocean Parkway</x:v>
+        <x:v>Garibaldi Memorial</x:v>
       </x:c>
       <x:c r="E16" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="F16" s="9" t="str">
-        <x:v>Wave Hill</x:v>
+        <x:v>Riverside Park and Drive</x:v>
       </x:c>
       <x:c r="G16" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H16" s="9" t="str">
-        <x:v>First Reformed Church of College Point</x:v>
+        <x:v>Whitney Museum of American Art (NY Studio School)</x:v>
       </x:c>
       <x:c r="I16" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J16" s="9" t="str">
-        <x:v>Moore-McMillen House</x:v>
+        <x:v>Flushing Armory</x:v>
       </x:c>
       <x:c r="K16" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L16" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -952,28 +952,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>High Bridge Aqueduct and Water Tower</x:v>
+        <x:v>Fort Tompkins Quadrangle</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="F17" s="9" t="str">
-        <x:v>Prospect Park Boathouse</x:v>
+        <x:v>Ocean Parkway</x:v>
       </x:c>
       <x:c r="G17" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H17" s="9" t="str">
-        <x:v>Flushing High School</x:v>
+        <x:v>New Dorp Light</x:v>
       </x:c>
       <x:c r="I17" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J17" s="9" t="str">
-        <x:v>Kreischer House</x:v>
+        <x:v>Candler Building</x:v>
       </x:c>
       <x:c r="K17" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L17" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -991,28 +991,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>Fort Wadsworth</x:v>
+        <x:v>Theodore Roosevelt Birthplace</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F18" s="9" t="str">
-        <x:v>Steinway House</x:v>
+        <x:v>Wave Hill</x:v>
       </x:c>
       <x:c r="G18" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H18" s="9" t="str">
-        <x:v>Nassau Brewery</x:v>
+        <x:v>Mary A. Whalen</x:v>
       </x:c>
       <x:c r="I18" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J18" s="9" t="str">
-        <x:v>Valentine-Varian House</x:v>
+        <x:v>Moore-McMillen House</x:v>
       </x:c>
       <x:c r="K18" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L18" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1030,28 +1030,28 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>The Public Theater</x:v>
+        <x:v>High Bridge Aqueduct and Water Tower</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="F19" s="9" t="str">
-        <x:v>Ward, Caleb T., Mansion</x:v>
+        <x:v>Prospect Park Boathouse</x:v>
       </x:c>
       <x:c r="G19" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H19" s="9" t="str">
-        <x:v>Brooklyn Trust Company</x:v>
+        <x:v>Columbus Monument</x:v>
       </x:c>
       <x:c r="I19" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J19" s="9" t="str">
-        <x:v>Grace Episcopal Church</x:v>
+        <x:v>Cary Building</x:v>
       </x:c>
       <x:c r="K19" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L19" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1069,28 +1069,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>Gracie Mansion</x:v>
+        <x:v>Fort Wadsworth</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="F20" s="9" t="str">
-        <x:v>Rego Park Jewish Center</x:v>
+        <x:v>Jeffrey's Hook Lighthouse</x:v>
       </x:c>
       <x:c r="G20" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H20" s="9" t="str">
-        <x:v>United Workers' Cooperatives</x:v>
+        <x:v>Casemate Fort, Whiting Quadrangle</x:v>
       </x:c>
       <x:c r="I20" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J20" s="9" t="str">
-        <x:v>LaTourette House</x:v>
+        <x:v>City &amp; Suburban Homes Company's York Avenue Estate</x:v>
       </x:c>
       <x:c r="K20" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L20" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1108,28 +1108,28 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>Riverside Park and Drive</x:v>
+        <x:v>Steinway House</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F21" s="9" t="str">
-        <x:v>Voorlezer's House</x:v>
+        <x:v>Ward, Caleb T., Mansion</x:v>
       </x:c>
       <x:c r="G21" s="9" t="str">
         <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H21" s="9" t="str">
-        <x:v>Bronx County Courthouse</x:v>
+        <x:v>Silver Lake Cemetery</x:v>
       </x:c>
       <x:c r="I21" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="J21" s="9" t="str">
-        <x:v>Trinity Lutheran Church</x:v>
+        <x:v>Kreischer House</x:v>
       </x:c>
       <x:c r="K21" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L21" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1147,28 +1147,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>Loew's Kameo Theater</x:v>
+        <x:v>African Burial Ground</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F22" s="9" t="str">
-        <x:v>Parkway Village</x:v>
+        <x:v>Rego Park Jewish Center</x:v>
       </x:c>
       <x:c r="G22" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="H22" s="9" t="str">
-        <x:v>St. Peter's Church, Chapel and Cemetery Complex</x:v>
+        <x:v>Appellate Division Courthouse of New York State</x:v>
       </x:c>
       <x:c r="I22" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J22" s="9" t="str">
-        <x:v>Boardman- Mitchell House</x:v>
+        <x:v>Lincoln Club</x:v>
       </x:c>
       <x:c r="K22" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="L22" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1186,25 +1186,25 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>McGolrick, Monsignor, Park and Shelter Pavilion</x:v>
+        <x:v>Loew's Kameo Theater</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F23" s="9" t="str">
-        <x:v>Old Town of Flushing Burial Ground</x:v>
+        <x:v>Ed Sullivan Theater</x:v>
       </x:c>
       <x:c r="G23" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H23" s="9" t="str">
-        <x:v>West Bank Light Station</x:v>
+        <x:v>University Settlement House</x:v>
       </x:c>
       <x:c r="I23" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J23" s="9" t="str">
-        <x:v>Riverdale Presbyterian Church Complex</x:v>
+        <x:v>Dodge, William E., House</x:v>
       </x:c>
       <x:c r="K23" s="9" t="str">
         <x:v>The Bronx</x:v>
@@ -1225,28 +1225,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>Eastern Parkway</x:v>
+        <x:v>Voorlezer's House</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="F24" s="9" t="str">
-        <x:v>RKO Keith's Theater</x:v>
+        <x:v>Hamilton Grange National Memorial</x:v>
       </x:c>
       <x:c r="G24" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H24" s="9" t="str">
-        <x:v>Keeper's House, Williamsbridge Reservoir</x:v>
+        <x:v>Beth-El Jewish Center of Flatbush</x:v>
       </x:c>
       <x:c r="I24" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J24" s="9" t="str">
-        <x:v>McFarlane-Bredt House</x:v>
+        <x:v>Congregation Tifereth Israel</x:v>
       </x:c>
       <x:c r="K24" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="L24" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1264,28 +1264,28 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>Theodore Roosevelt Birthplace</x:v>
+        <x:v>New York Public Library</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F25" s="9" t="str">
-        <x:v>Loew's King Theatre</x:v>
+        <x:v>Parkway Village</x:v>
       </x:c>
       <x:c r="G25" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H25" s="9" t="str">
-        <x:v>Ward's Point Conservation Area</x:v>
+        <x:v>Gage and Tollner Restaurant</x:v>
       </x:c>
       <x:c r="I25" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J25" s="9" t="str">
-        <x:v>C. Rieger's Sons Factory</x:v>
+        <x:v>Spear &amp; Company Factory</x:v>
       </x:c>
       <x:c r="K25" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L25" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1303,28 +1303,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>Crotona Play Center</x:v>
+        <x:v>McGolrick, Monsignor, Park and Shelter Pavilion</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F26" s="9" t="str">
-        <x:v>Parkway Theater</x:v>
+        <x:v>Morgan Library</x:v>
       </x:c>
       <x:c r="G26" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H26" s="9" t="str">
-        <x:v>Maple Grove Cemetery</x:v>
+        <x:v>Lighthouse</x:v>
       </x:c>
       <x:c r="I26" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J26" s="9" t="str">
-        <x:v>Kreuzer-Pelton House</x:v>
+        <x:v>Cornell Farmhouse</x:v>
       </x:c>
       <x:c r="K26" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L26" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1342,25 +1342,25 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>Jeffrey's Hook Lighthouse</x:v>
+        <x:v>Old Town of Flushing Burial Ground</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F27" s="9" t="str">
-        <x:v>Flushing Town Hall</x:v>
+        <x:v>Eastern Parkway</x:v>
       </x:c>
       <x:c r="G27" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H27" s="9" t="str">
-        <x:v>Boston Road Plaza</x:v>
+        <x:v>DeLamar Mansion</x:v>
       </x:c>
       <x:c r="I27" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J27" s="9" t="str">
-        <x:v>Immanuel Union Church</x:v>
+        <x:v>LaTourette House</x:v>
       </x:c>
       <x:c r="K27" s="9" t="str">
         <x:v>Staten Island</x:v>
@@ -1381,28 +1381,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>B &amp; B Carousell</x:v>
+        <x:v>Trinity Church and Graveyard</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F28" s="9" t="str">
-        <x:v>Fort Schuyler</x:v>
+        <x:v>RKO Keith's Theater</x:v>
       </x:c>
       <x:c r="G28" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="H28" s="9" t="str">
-        <x:v>Queens County Savings Bank, Kew Gardens Hills Branch</x:v>
+        <x:v>Casita Rincon Criollo</x:v>
       </x:c>
       <x:c r="I28" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J28" s="9" t="str">
-        <x:v>Christ Church New Brighton</x:v>
+        <x:v>Bayard-Condict Building</x:v>
       </x:c>
       <x:c r="K28" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L28" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1420,28 +1420,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>U.S. Army Military Ocean Terminal</x:v>
+        <x:v>Loew's King Theatre</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F29" s="9" t="str">
-        <x:v>Old Orchard Shoal Light Station</x:v>
+        <x:v>Crotona Play Center</x:v>
       </x:c>
       <x:c r="G29" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H29" s="9" t="str">
-        <x:v>Office of the Register</x:v>
+        <x:v>Trinity Chapel</x:v>
       </x:c>
       <x:c r="I29" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J29" s="9" t="str">
-        <x:v>Reformed Church of Melrose</x:v>
+        <x:v>New York Congregational Home for the Aged</x:v>
       </x:c>
       <x:c r="K29" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="L29" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1459,28 +1459,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>Ocean Parkway Jewish Center</x:v>
+        <x:v>Castle Clinton National Monument</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F30" s="9" t="str">
-        <x:v>Staten Island Ferry Terminal</x:v>
+        <x:v>Queensboro Bridge</x:v>
       </x:c>
       <x:c r="G30" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H30" s="9" t="str">
-        <x:v>Long Island City Courthouse Complex</x:v>
+        <x:v>First Reformed Church of College Point</x:v>
       </x:c>
       <x:c r="I30" s="9" t="str">
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="J30" s="9" t="str">
-        <x:v>St. Anselm's Roman Catholic Church Complex</x:v>
+        <x:v>Trinity Lutheran Church</x:v>
       </x:c>
       <x:c r="K30" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L30" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1498,28 +1498,28 @@
         <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>African Burial Ground</x:v>
+        <x:v>Parkway Theater</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F31" s="9" t="str">
-        <x:v>Long Island Motor Parkway</x:v>
+        <x:v>B &amp; B Carousell</x:v>
       </x:c>
       <x:c r="G31" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H31" s="9" t="str">
-        <x:v>Mary A. Whalen</x:v>
+        <x:v>Joralemon Street Tunnel (IRT)</x:v>
       </x:c>
       <x:c r="I31" s="9" t="str">
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J31" s="9" t="str">
-        <x:v>Louis A. and Laura Stirn House</x:v>
+        <x:v>Decker Building</x:v>
       </x:c>
       <x:c r="K31" s="9" t="str">
-        <x:v>Staten Island</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="L31" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1537,28 +1537,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>Ed Sullivan Theater</x:v>
+        <x:v>Flushing Town Hall</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F32" s="9" t="str">
-        <x:v>Hamilton Grange National Memorial</x:v>
+        <x:v>U.S. Army Military Ocean Terminal</x:v>
       </x:c>
       <x:c r="G32" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="H32" s="9" t="str">
-        <x:v>Casemate Fort, Whiting Quadrangle</x:v>
+        <x:v>Ottendorfer Public Library and Stuyvesant Polyclinic Hospital</x:v>
       </x:c>
       <x:c r="I32" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J32" s="9" t="str">
-        <x:v>Conrad Voelcker House</x:v>
+        <x:v>English Evangelical Lutheran Church of the Reformation</x:v>
       </x:c>
       <x:c r="K32" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="L32" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1576,28 +1576,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>New York Public Library</x:v>
+        <x:v>American Stock Exchange</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F33" s="9" t="str">
-        <x:v>Morgan Library</x:v>
+        <x:v>Fort Schuyler</x:v>
       </x:c>
       <x:c r="G33" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="H33" s="9" t="str">
-        <x:v>Beth-El Jewish Center of Flatbush</x:v>
+        <x:v>Sheffield Farms Stable</x:v>
       </x:c>
       <x:c r="I33" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="J33" s="9" t="str">
-        <x:v>Sohmer Piano Factory</x:v>
+        <x:v>Boardman- Mitchell House</x:v>
       </x:c>
       <x:c r="K33" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L33" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1615,28 +1615,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>Trinity Church and Graveyard</x:v>
+        <x:v>Ocean Parkway Jewish Center</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="F34" s="9" t="str">
-        <x:v>Castle Clinton National Monument</x:v>
+        <x:v>Old Orchard Shoal Light Station</x:v>
       </x:c>
       <x:c r="G34" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H34" s="9" t="str">
-        <x:v>Gage and Tollner Restaurant</x:v>
+        <x:v>Flushing High School</x:v>
       </x:c>
       <x:c r="I34" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="J34" s="9" t="str">
-        <x:v>Saint James Church</x:v>
+        <x:v>Valentine-Varian House</x:v>
       </x:c>
       <x:c r="K34" s="9" t="str">
-        <x:v>Queens</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="L34" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1654,28 +1654,28 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>Queensboro Bridge</x:v>
+        <x:v>Whitney Museum of American Art</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="F35" s="9" t="str">
-        <x:v>American Stock Exchange</x:v>
+        <x:v>Staten Island Ferry Terminal</x:v>
       </x:c>
       <x:c r="G35" s="9" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="H35" s="9" t="str">
-        <x:v>Joralemon Street Tunnel (IRT)</x:v>
+        <x:v>United Workers' Cooperatives</x:v>
       </x:c>
       <x:c r="I35" s="9" t="str">
-        <x:v>Brooklyn</x:v>
+        <x:v>The Bronx</x:v>
       </x:c>
       <x:c r="J35" s="9" t="str">
-        <x:v>Spaulding, Henry F., Coachman's House</x:v>
+        <x:v>Conrad Voelcker House</x:v>
       </x:c>
       <x:c r="K35" s="9" t="str">
-        <x:v>The Bronx</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="L35" s="16" t="str">
         <x:v>scheduled</x:v>
@@ -1693,10 +1693,10 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="D36" s="11" t="str">
-        <x:v>Whitney Museum of American Art</x:v>
+        <x:v>Long Island Motor Parkway</x:v>
       </x:c>
       <x:c r="E36" s="11" t="str">
-        <x:v>Manhattan</x:v>
+        <x:v>Queens</x:v>
       </x:c>
       <x:c r="F36" s="11" t="str">
         <x:v>College of the City of New York</x:v>
@@ -1711,10 +1711,10 @@
         <x:v>Brooklyn</x:v>
       </x:c>
       <x:c r="J36" s="11" t="str">
-        <x:v>Jamaica Savings Bank</x:v>
+        <x:v>McFarlane-Bredt House</x:v>
       </x:c>
       <x:c r="K36" s="11" t="str">
-        <x:v>Queens</x:v>
+        <x:v>Staten Island</x:v>
       </x:c>
       <x:c r="L36" s="17" t="str">
         <x:v>scheduled</x:v>

</xml_diff>

<commit_message>
Add Wikipedia reveal previews
</commit_message>
<xml_diff>
--- a/exports/daily-games.xlsx
+++ b/exports/daily-games.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Games" sheetId="1" r:id="R27a0945120064f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Locations" sheetId="2" r:id="Rfc0846ec19494109"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog Summary" sheetId="3" r:id="Raad1979b850d4996"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dedupe Review" sheetId="4" r:id="Raf7a4a216f65409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Games" sheetId="1" r:id="R466b08c82aff479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Locations" sheetId="2" r:id="Rbaac8aed3c6b4409"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog Summary" sheetId="3" r:id="R1a4046e0dd7a456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dedupe Review" sheetId="4" r:id="Rb3bfeb887b704569"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -893,10 +893,10 @@
         <x:v>Queens</x:v>
       </x:c>
       <x:c r="H2" s="85" t="str">
-        <x:v>loc-0452</x:v>
+        <x:v>loc-0469</x:v>
       </x:c>
       <x:c r="I2" s="85" t="str">
-        <x:v>Trump Tower</x:v>
+        <x:v>Bank of America Tower</x:v>
       </x:c>
       <x:c r="J2" s="85" t="str">
         <x:v>Manhattan</x:v>
@@ -1217,10 +1217,10 @@
         <x:v>Manhattan</x:v>
       </x:c>
       <x:c r="H8" s="85" t="str">
-        <x:v>loc-0469</x:v>
+        <x:v>loc-0452</x:v>
       </x:c>
       <x:c r="I8" s="85" t="str">
-        <x:v>Bank of America Tower</x:v>
+        <x:v>Trump Tower</x:v>
       </x:c>
       <x:c r="J8" s="85" t="str">
         <x:v>Manhattan</x:v>
@@ -4923,7 +4923,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3faaed5333f4bf4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55fe259df43046df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -23803,7 +23803,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab095198ca0f4118"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1792a3ebb2734274"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27445,7 +27445,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf657f4dec6ab4182"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66f6f4c860574a05"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>